<commit_message>
swapping CMOS command order so remove_all_data is less risky
</commit_message>
<xml_diff>
--- a/commands/cmos1/cmos1_command_deck.xlsx
+++ b/commands/cmos1/cmos1_command_deck.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thanasi/Documents/FOXSI/GSE/GSE-FOXSI-4/foxsi4-commands/commands/cmos1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D5C583-1720-A54B-BBCE-B597A1043A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06AAA3E8-7C74-7F4E-8F76-8507655277A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="760" windowWidth="30220" windowHeight="17880" xr2:uid="{1DE950B2-129E-5A4D-8896-FB78BBCF4CAC}"/>
+    <workbookView xWindow="20" yWindow="760" windowWidth="30220" windowHeight="17820" xr2:uid="{1DE950B2-129E-5A4D-8896-FB78BBCF4CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="all_systems" sheetId="1" r:id="rId1"/>
@@ -1060,7 +1060,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1128,14 +1128,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1154,9 +1146,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1194,7 +1186,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1300,7 +1292,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1442,7 +1434,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1470,8 +1462,8 @@
     <col min="25" max="25" width="12.83203125" style="20" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11.1640625" style="20" customWidth="1"/>
     <col min="27" max="27" width="27.6640625" style="21" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5.5" style="42" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.1640625" style="42" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="5.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.1640625" style="20" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="19.1640625" customWidth="1"/>
     <col min="31" max="31" width="73.1640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1514,8 +1506,8 @@
       </c>
       <c r="Z1" s="35"/>
       <c r="AA1" s="36"/>
-      <c r="AB1" s="37"/>
-      <c r="AC1" s="37"/>
+      <c r="AB1" s="2"/>
+      <c r="AC1" s="2"/>
     </row>
     <row r="2" spans="1:31" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -1599,10 +1591,10 @@
       <c r="AA2" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="AB2" s="38" t="s">
+      <c r="AB2" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="AC2" s="38" t="s">
+      <c r="AC2" s="1" t="s">
         <v>299</v>
       </c>
       <c r="AD2" s="1" t="s">
@@ -1695,7 +1687,7 @@
       <c r="AA3" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB3" s="39">
+      <c r="AB3" s="27">
         <v>71</v>
       </c>
       <c r="AC3" s="27" t="s">
@@ -1791,7 +1783,7 @@
       <c r="AA4" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB4" s="39">
+      <c r="AB4" s="27">
         <v>72</v>
       </c>
       <c r="AC4" s="27" t="s">
@@ -1887,7 +1879,7 @@
       <c r="AA5" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB5" s="39">
+      <c r="AB5" s="27">
         <v>73</v>
       </c>
       <c r="AC5" s="27" t="s">
@@ -1983,7 +1975,7 @@
       <c r="AA6" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB6" s="39">
+      <c r="AB6" s="27">
         <v>44</v>
       </c>
       <c r="AC6" s="27" t="s">
@@ -2079,7 +2071,7 @@
       <c r="AA7" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB7" s="39">
+      <c r="AB7" s="27">
         <v>45</v>
       </c>
       <c r="AC7" s="27" t="s">
@@ -2175,7 +2167,7 @@
       <c r="AA8" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB8" s="39">
+      <c r="AB8" s="27">
         <v>46</v>
       </c>
       <c r="AC8" s="27" t="s">
@@ -2271,7 +2263,7 @@
       <c r="AA9" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB9" s="39">
+      <c r="AB9" s="27">
         <v>47</v>
       </c>
       <c r="AC9" s="27" t="s">
@@ -2367,7 +2359,7 @@
       <c r="AA10" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB10" s="39">
+      <c r="AB10" s="27">
         <v>48</v>
       </c>
       <c r="AC10" s="27" t="s">
@@ -2463,7 +2455,7 @@
       <c r="AA11" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB11" s="39">
+      <c r="AB11" s="27">
         <v>49</v>
       </c>
       <c r="AC11" s="27" t="s">
@@ -2559,7 +2551,7 @@
       <c r="AA12" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB12" s="39">
+      <c r="AB12" s="27">
         <v>50</v>
       </c>
       <c r="AC12" s="27" t="s">
@@ -2655,7 +2647,7 @@
       <c r="AA13" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB13" s="39">
+      <c r="AB13" s="27">
         <v>51</v>
       </c>
       <c r="AC13" s="27" t="s">
@@ -2751,7 +2743,7 @@
       <c r="AA14" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB14" s="39">
+      <c r="AB14" s="27">
         <v>52</v>
       </c>
       <c r="AC14" s="27" t="s">
@@ -2847,7 +2839,7 @@
       <c r="AA15" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB15" s="39">
+      <c r="AB15" s="27">
         <v>53</v>
       </c>
       <c r="AC15" s="27" t="s">
@@ -2943,7 +2935,7 @@
       <c r="AA16" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB16" s="39">
+      <c r="AB16" s="27">
         <v>54</v>
       </c>
       <c r="AC16" s="27" t="s">
@@ -3039,7 +3031,7 @@
       <c r="AA17" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB17" s="39">
+      <c r="AB17" s="27">
         <v>55</v>
       </c>
       <c r="AC17" s="27" t="s">
@@ -3135,7 +3127,7 @@
       <c r="AA18" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB18" s="39">
+      <c r="AB18" s="27">
         <v>56</v>
       </c>
       <c r="AC18" s="27" t="s">
@@ -3231,7 +3223,7 @@
       <c r="AA19" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB19" s="39">
+      <c r="AB19" s="27">
         <v>57</v>
       </c>
       <c r="AC19" s="27" t="s">
@@ -3327,7 +3319,7 @@
       <c r="AA20" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB20" s="39">
+      <c r="AB20" s="27">
         <v>58</v>
       </c>
       <c r="AC20" s="27" t="s">
@@ -3423,7 +3415,7 @@
       <c r="AA21" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB21" s="39">
+      <c r="AB21" s="27">
         <v>59</v>
       </c>
       <c r="AC21" s="27" t="s">
@@ -3519,7 +3511,7 @@
       <c r="AA22" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB22" s="39">
+      <c r="AB22" s="27">
         <v>60</v>
       </c>
       <c r="AC22" s="27" t="s">
@@ -3615,7 +3607,7 @@
       <c r="AA23" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB23" s="39">
+      <c r="AB23" s="27">
         <v>61</v>
       </c>
       <c r="AC23" s="27" t="s">
@@ -3711,7 +3703,7 @@
       <c r="AA24" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB24" s="39">
+      <c r="AB24" s="27">
         <v>62</v>
       </c>
       <c r="AC24" s="27" t="s">
@@ -3807,7 +3799,7 @@
       <c r="AA25" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB25" s="39">
+      <c r="AB25" s="27">
         <v>63</v>
       </c>
       <c r="AC25" s="27" t="s">
@@ -3903,7 +3895,7 @@
       <c r="AA26" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB26" s="39">
+      <c r="AB26" s="27">
         <v>64</v>
       </c>
       <c r="AC26" s="27" t="s">
@@ -3999,7 +3991,7 @@
       <c r="AA27" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB27" s="39">
+      <c r="AB27" s="27">
         <v>65</v>
       </c>
       <c r="AC27" s="27" t="s">
@@ -4095,7 +4087,7 @@
       <c r="AA28" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB28" s="39">
+      <c r="AB28" s="27">
         <v>66</v>
       </c>
       <c r="AC28" s="27" t="s">
@@ -4191,7 +4183,7 @@
       <c r="AA29" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB29" s="39">
+      <c r="AB29" s="27">
         <v>67</v>
       </c>
       <c r="AC29" s="27" t="s">
@@ -4287,7 +4279,7 @@
       <c r="AA30" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB30" s="39">
+      <c r="AB30" s="27">
         <v>68</v>
       </c>
       <c r="AC30" s="27" t="s">
@@ -4383,7 +4375,7 @@
       <c r="AA31" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB31" s="39">
+      <c r="AB31" s="27">
         <v>69</v>
       </c>
       <c r="AC31" s="27" t="s">
@@ -4479,7 +4471,7 @@
       <c r="AA32" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="AB32" s="39">
+      <c r="AB32" s="27">
         <v>70</v>
       </c>
       <c r="AC32" s="27" t="s">
@@ -4519,8 +4511,8 @@
       <c r="Y33" s="24"/>
       <c r="Z33" s="7"/>
       <c r="AA33" s="24"/>
-      <c r="AB33" s="41"/>
-      <c r="AC33" s="41"/>
+      <c r="AB33" s="7"/>
+      <c r="AC33" s="7"/>
     </row>
     <row r="34" spans="1:31" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
@@ -4605,7 +4597,7 @@
       <c r="AA34" s="23">
         <v>0</v>
       </c>
-      <c r="AB34" s="40">
+      <c r="AB34" s="3">
         <v>74</v>
       </c>
       <c r="AC34" s="27" t="s">
@@ -4701,7 +4693,7 @@
       <c r="AA35" s="23">
         <v>0</v>
       </c>
-      <c r="AB35" s="40">
+      <c r="AB35" s="3">
         <v>75</v>
       </c>
       <c r="AC35" s="27" t="s">
@@ -4797,8 +4789,8 @@
       <c r="AA36" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB36" s="40">
-        <v>7</v>
+      <c r="AB36" s="3">
+        <v>6</v>
       </c>
       <c r="AC36" s="27" t="s">
         <v>301</v>
@@ -4893,8 +4885,8 @@
       <c r="AA37" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB37" s="40">
-        <v>8</v>
+      <c r="AB37" s="3">
+        <v>7</v>
       </c>
       <c r="AC37" s="27" t="s">
         <v>301</v>
@@ -4989,8 +4981,8 @@
       <c r="AA38" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB38" s="40">
-        <v>9</v>
+      <c r="AB38" s="3">
+        <v>8</v>
       </c>
       <c r="AC38" s="27" t="s">
         <v>301</v>
@@ -5085,7 +5077,7 @@
       <c r="AA39" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="AB39" s="40">
+      <c r="AB39" s="3">
         <v>82</v>
       </c>
       <c r="AC39" s="27" t="s">
@@ -5181,8 +5173,8 @@
       <c r="AA40" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB40" s="40">
-        <v>10</v>
+      <c r="AB40" s="3">
+        <v>9</v>
       </c>
       <c r="AC40" s="27" t="s">
         <v>301</v>
@@ -5277,7 +5269,7 @@
       <c r="AA41" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB41" s="40">
+      <c r="AB41" s="3">
         <v>2</v>
       </c>
       <c r="AC41" s="27" t="s">
@@ -5373,7 +5365,7 @@
       <c r="AA42" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB42" s="40">
+      <c r="AB42" s="3">
         <v>1</v>
       </c>
       <c r="AC42" s="27" t="s">
@@ -5469,10 +5461,10 @@
       <c r="AA43" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB43" s="40">
+      <c r="AB43" s="3">
         <v>3</v>
       </c>
-      <c r="AC43" s="40" t="s">
+      <c r="AC43" s="3" t="s">
         <v>302</v>
       </c>
       <c r="AD43" t="s">
@@ -5565,8 +5557,8 @@
       <c r="AA44" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB44" s="40">
-        <v>5</v>
+      <c r="AB44" s="3">
+        <v>4</v>
       </c>
       <c r="AC44" s="27" t="s">
         <v>301</v>
@@ -5661,8 +5653,8 @@
       <c r="AA45" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB45" s="40">
-        <v>6</v>
+      <c r="AB45" s="3">
+        <v>5</v>
       </c>
       <c r="AC45" s="27" t="s">
         <v>301</v>
@@ -5757,8 +5749,8 @@
       <c r="AA46" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB46" s="40">
-        <v>4</v>
+      <c r="AB46" s="3">
+        <v>10</v>
       </c>
       <c r="AC46" s="27" t="s">
         <v>300</v>
@@ -5853,7 +5845,7 @@
       <c r="AA47" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB47" s="40">
+      <c r="AB47" s="3">
         <v>11</v>
       </c>
       <c r="AC47" s="27" t="s">
@@ -5949,7 +5941,7 @@
       <c r="AA48" s="23" t="s">
         <v>251</v>
       </c>
-      <c r="AB48" s="40">
+      <c r="AB48" s="3">
         <v>12</v>
       </c>
       <c r="AC48" s="27" t="s">
@@ -6045,7 +6037,7 @@
       <c r="AA49" s="23" t="s">
         <v>252</v>
       </c>
-      <c r="AB49" s="40">
+      <c r="AB49" s="3">
         <v>13</v>
       </c>
       <c r="AC49" s="27" t="s">
@@ -6141,7 +6133,7 @@
       <c r="AA50" s="23" t="s">
         <v>253</v>
       </c>
-      <c r="AB50" s="40">
+      <c r="AB50" s="3">
         <v>14</v>
       </c>
       <c r="AC50" s="27" t="s">
@@ -6237,7 +6229,7 @@
       <c r="AA51" s="23" t="s">
         <v>254</v>
       </c>
-      <c r="AB51" s="40">
+      <c r="AB51" s="3">
         <v>15</v>
       </c>
       <c r="AC51" s="27" t="s">
@@ -6333,7 +6325,7 @@
       <c r="AA52" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="AB52" s="40">
+      <c r="AB52" s="3">
         <v>16</v>
       </c>
       <c r="AC52" s="27" t="s">
@@ -6429,7 +6421,7 @@
       <c r="AA53" s="25" t="s">
         <v>256</v>
       </c>
-      <c r="AB53" s="40">
+      <c r="AB53" s="3">
         <v>17</v>
       </c>
       <c r="AC53" s="27" t="s">
@@ -6525,7 +6517,7 @@
       <c r="AA54" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="AB54" s="40">
+      <c r="AB54" s="3">
         <v>18</v>
       </c>
       <c r="AC54" s="27" t="s">
@@ -6621,7 +6613,7 @@
       <c r="AA55" s="25" t="s">
         <v>258</v>
       </c>
-      <c r="AB55" s="40">
+      <c r="AB55" s="3">
         <v>19</v>
       </c>
       <c r="AC55" s="27" t="s">
@@ -6717,7 +6709,7 @@
       <c r="AA56" s="25" t="s">
         <v>259</v>
       </c>
-      <c r="AB56" s="40">
+      <c r="AB56" s="3">
         <v>20</v>
       </c>
       <c r="AC56" s="27" t="s">
@@ -6813,7 +6805,7 @@
       <c r="AA57" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="AB57" s="40">
+      <c r="AB57" s="3">
         <v>21</v>
       </c>
       <c r="AC57" s="27" t="s">
@@ -6909,7 +6901,7 @@
       <c r="AA58" s="23" t="s">
         <v>261</v>
       </c>
-      <c r="AB58" s="40">
+      <c r="AB58" s="3">
         <v>22</v>
       </c>
       <c r="AC58" s="27" t="s">
@@ -7005,7 +6997,7 @@
       <c r="AA59" s="25" t="s">
         <v>262</v>
       </c>
-      <c r="AB59" s="40">
+      <c r="AB59" s="3">
         <v>23</v>
       </c>
       <c r="AC59" s="27" t="s">
@@ -7101,7 +7093,7 @@
       <c r="AA60" s="25" t="s">
         <v>263</v>
       </c>
-      <c r="AB60" s="40">
+      <c r="AB60" s="3">
         <v>24</v>
       </c>
       <c r="AC60" s="27" t="s">
@@ -7197,7 +7189,7 @@
       <c r="AA61" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="AB61" s="40">
+      <c r="AB61" s="3">
         <v>25</v>
       </c>
       <c r="AC61" s="27" t="s">
@@ -7293,7 +7285,7 @@
       <c r="AA62" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="AB62" s="40">
+      <c r="AB62" s="3">
         <v>26</v>
       </c>
       <c r="AC62" s="27" t="s">
@@ -7389,7 +7381,7 @@
       <c r="AA63" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="AB63" s="40">
+      <c r="AB63" s="3">
         <v>27</v>
       </c>
       <c r="AC63" s="27" t="s">
@@ -7485,7 +7477,7 @@
       <c r="AA64" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="AB64" s="40">
+      <c r="AB64" s="3">
         <v>28</v>
       </c>
       <c r="AC64" s="27" t="s">
@@ -7581,7 +7573,7 @@
       <c r="AA65" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="AB65" s="40">
+      <c r="AB65" s="3">
         <v>29</v>
       </c>
       <c r="AC65" s="27" t="s">
@@ -7677,7 +7669,7 @@
       <c r="AA66" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="AB66" s="40">
+      <c r="AB66" s="3">
         <v>30</v>
       </c>
       <c r="AC66" s="27" t="s">
@@ -7773,7 +7765,7 @@
       <c r="AA67" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="AB67" s="40">
+      <c r="AB67" s="3">
         <v>31</v>
       </c>
       <c r="AC67" s="27" t="s">
@@ -7869,7 +7861,7 @@
       <c r="AA68" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="AB68" s="40">
+      <c r="AB68" s="3">
         <v>32</v>
       </c>
       <c r="AC68" s="27" t="s">
@@ -7965,7 +7957,7 @@
       <c r="AA69" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="AB69" s="40">
+      <c r="AB69" s="3">
         <v>33</v>
       </c>
       <c r="AC69" s="27" t="s">
@@ -8061,7 +8053,7 @@
       <c r="AA70" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="AB70" s="40">
+      <c r="AB70" s="3">
         <v>34</v>
       </c>
       <c r="AC70" s="27" t="s">
@@ -8157,7 +8149,7 @@
       <c r="AA71" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="AB71" s="40">
+      <c r="AB71" s="3">
         <v>35</v>
       </c>
       <c r="AC71" s="27" t="s">
@@ -8253,7 +8245,7 @@
       <c r="AA72" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="AB72" s="40">
+      <c r="AB72" s="3">
         <v>36</v>
       </c>
       <c r="AC72" s="27" t="s">
@@ -8349,7 +8341,7 @@
       <c r="AA73" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="AB73" s="40">
+      <c r="AB73" s="3">
         <v>37</v>
       </c>
       <c r="AC73" s="27" t="s">
@@ -8445,7 +8437,7 @@
       <c r="AA74" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="AB74" s="40">
+      <c r="AB74" s="3">
         <v>38</v>
       </c>
       <c r="AC74" s="27" t="s">
@@ -8541,7 +8533,7 @@
       <c r="AA75" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="AB75" s="40">
+      <c r="AB75" s="3">
         <v>39</v>
       </c>
       <c r="AC75" s="27" t="s">
@@ -8637,7 +8629,7 @@
       <c r="AA76" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="AB76" s="40">
+      <c r="AB76" s="3">
         <v>40</v>
       </c>
       <c r="AC76" s="27" t="s">
@@ -8733,7 +8725,7 @@
       <c r="AA77" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="AB77" s="40">
+      <c r="AB77" s="3">
         <v>41</v>
       </c>
       <c r="AC77" s="27" t="s">
@@ -8829,7 +8821,7 @@
       <c r="AA78" s="23" t="s">
         <v>264</v>
       </c>
-      <c r="AB78" s="40">
+      <c r="AB78" s="3">
         <v>42</v>
       </c>
       <c r="AC78" s="27" t="s">
@@ -8925,7 +8917,7 @@
       <c r="AA79" s="23" t="s">
         <v>264</v>
       </c>
-      <c r="AB79" s="40">
+      <c r="AB79" s="3">
         <v>43</v>
       </c>
       <c r="AC79" s="27" t="s">
@@ -9021,7 +9013,7 @@
       <c r="AA80" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB80" s="40">
+      <c r="AB80" s="3">
         <v>76</v>
       </c>
       <c r="AC80" s="27" t="s">
@@ -9117,7 +9109,7 @@
       <c r="AA81" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB81" s="40">
+      <c r="AB81" s="3">
         <v>77</v>
       </c>
       <c r="AC81" s="27" t="s">
@@ -9213,7 +9205,7 @@
       <c r="AA82" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB82" s="40">
+      <c r="AB82" s="3">
         <v>78</v>
       </c>
       <c r="AC82" s="27" t="s">
@@ -9309,7 +9301,7 @@
       <c r="AA83" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB83" s="40">
+      <c r="AB83" s="3">
         <v>79</v>
       </c>
       <c r="AC83" s="27" t="s">
@@ -9405,7 +9397,7 @@
       <c r="AA84" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB84" s="40">
+      <c r="AB84" s="3">
         <v>80</v>
       </c>
       <c r="AC84" s="27" t="s">
@@ -9501,7 +9493,7 @@
       <c r="AA85" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="AB85" s="40">
+      <c r="AB85" s="3">
         <v>81</v>
       </c>
       <c r="AC85" s="27" t="s">

</xml_diff>